<commit_message>
Graphes du cockpit : 6 mini-graphes KPI + graphe de tendance dans la feuille
- Feuille Cockpit : ajout de 6 mini-graphes (sparkline-style, une courbe 3 ans
  par KPI) + le graphe de tendance base 100 (Activité vs Dépenses). 7 objets
  graphiques au total, de vrais charts Excel reproductibles nativement.
- Décision figée : le graphe de tendance vit DANS le cockpit (plus de rapport
  Tendance séparé). Guide de dev mis à jour (T3 fusionné dans T1, ordre revu).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/MAQUETTES_RAPPORTS.xlsx
+++ b/eduservices/tagetik/MAQUETTES_RAPPORTS.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -164,6 +164,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000A5A48"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000A5A48"/>
       <sz val="10"/>
     </font>
@@ -236,10 +242,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -265,6 +271,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -483,7 +490,505 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Activité vs Dépenses d'acquisition (base 100)</a:t>
+              <a:t>Chiffre d'affaires (€)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$11:$D$11</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>EBITDA (€)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$12:$D$12</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Marge EBITDA %</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$13:$D$13</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Leads</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$14:$D$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Inscrits</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$15:$D$15</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>CAC (€/inscrit)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$10:$D$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$16:$D$16</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tendance base 100 : Activité (CA) vs Dépenses d'acquisition</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -600,7 +1105,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="2520000"/>
+    <ext cx="2376000" cy="936000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -610,6 +1115,138 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2376000" cy="936000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2376000" cy="936000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2376000" cy="936000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2376000" cy="936000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2376000" cy="936000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1079,7 +1716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1178,141 +1815,146 @@
           <t>YoY 25→26</t>
         </is>
       </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>GRAPHES KPI  (sparklines 3 ans)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Chiffre d'affaires (€)</t>
         </is>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="16">
         <f>SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="16">
         <f>SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="16">
         <f>SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="17">
         <f>IFERROR((D11-C11)/C11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>EBITDA (€)</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>(SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <f>(SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>(SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="17">
         <f>IFERROR((D12-C12)/C12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Marge EBITDA %</t>
         </is>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="18">
         <f>(SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))/SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="18">
         <f>(SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))/SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="18">
         <f>(SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES"))/SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="19">
         <f>D13-C13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <f>SUM('Données CRM'!C5:C9)</f>
         <v/>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <f>SUM('Données CRM'!C10:C14)</f>
         <v/>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <f>SUM('Données CRM'!C15:C19)</f>
         <v/>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="17">
         <f>IFERROR((D14-C14)/C14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <f>SUM('Données CRM'!F5:F9)</f>
         <v/>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <f>SUM('Données CRM'!F10:F14)</f>
         <v/>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <f>SUM('Données CRM'!F15:F19)</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="17">
         <f>IFERROR((D15-C15)/C15,0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>CAC (€/inscrit)</t>
         </is>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="21">
         <f>SUM('Données CRM'!H5:H9)/SUM('Données CRM'!F5:F9)</f>
         <v/>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="21">
         <f>SUM('Données CRM'!H10:H14)/SUM('Données CRM'!F10:F14)</f>
         <v/>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="21">
         <f>SUM('Données CRM'!H15:H19)/SUM('Données CRM'!F15:F19)</f>
         <v/>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="22">
         <f>IFERROR((D16-C16)/C16,0)</f>
         <v/>
       </c>
@@ -1325,62 +1967,62 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>TENDANCE — base 100 en 2024 (source V_TENDANCE)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Année</t>
         </is>
       </c>
-      <c r="B21" s="24" t="n">
+      <c r="B21" s="25" t="n">
         <v>2024</v>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="25" t="n">
         <v>2025</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="25" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Activité (CA)</t>
         </is>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="27">
         <f>B11/$B$11*100</f>
         <v/>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="27">
         <f>C11/$B$11*100</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="27">
         <f>D11/$B$11*100</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Dépenses acq.</t>
         </is>
       </c>
-      <c r="B23" s="26">
+      <c r="B23" s="27">
         <f>(SUM('Données CRM'!H5:H9))/(SUM('Données CRM'!H5:H9))*100</f>
         <v/>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="27">
         <f>(SUM('Données CRM'!H10:H14))/(SUM('Données CRM'!H5:H9))*100</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="27">
         <f>(SUM('Données CRM'!H15:H19))/(SUM('Données CRM'!H5:H9))*100</f>
         <v/>
       </c>
@@ -1429,235 +2071,235 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>en €</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E5" s="28" t="inlineStr">
+      <c r="E5" s="29" t="inlineStr">
         <is>
           <t>Δ 25→26</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="B6" s="30">
+      <c r="B6" s="31">
         <f>SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="31">
         <f>SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="D6" s="30">
+      <c r="D6" s="31">
         <f>SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PRODUITS")</f>
         <v/>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="32">
         <f>IFERROR((G6-F6)/F6,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>Coûts directs</t>
         </is>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <f>-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <f>-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")</f>
         <v/>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <f>-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"COUTS_DIRECTS")</f>
         <v/>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="22">
         <f>IFERROR((G7-F7)/F7,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Personnel</t>
         </is>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <f>-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")</f>
         <v/>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="16">
         <f>-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")</f>
         <v/>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="16">
         <f>-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"PERSONNEL")</f>
         <v/>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="22">
         <f>IFERROR((G8-F8)/F8,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t>Structure</t>
         </is>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <f>-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")</f>
         <v/>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <f>-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")</f>
         <v/>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="16">
         <f>-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"STRUCTURE")</f>
         <v/>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="22">
         <f>IFERROR((G9-F9)/F9,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Impôts &amp; taxes</t>
         </is>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="16">
         <f>-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES")</f>
         <v/>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="16">
         <f>-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES")</f>
         <v/>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="16">
         <f>-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"IMPOTS_TAXES")</f>
         <v/>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="22">
         <f>IFERROR((G10-F10)/F10,0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B11" s="34">
+      <c r="B11" s="35">
         <f>B6+SUM(B7:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="34">
+      <c r="C11" s="35">
         <f>C6+SUM(C7:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="34">
+      <c r="D11" s="35">
         <f>D6+SUM(D7:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="35">
+      <c r="E11" s="36">
         <f>IFERROR((G11-F11)/F11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Dotations (D&amp;A)</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>-SUMIFS('Données P&amp;L'!$E$5:$E$27,'Données P&amp;L'!$C$5:$C$27,"DOTATIONS")</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <f>-SUMIFS('Données P&amp;L'!$F$5:$F$27,'Données P&amp;L'!$C$5:$C$27,"DOTATIONS")</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>-SUMIFS('Données P&amp;L'!$G$5:$G$27,'Données P&amp;L'!$C$5:$C$27,"DOTATIONS")</f>
         <v/>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="22">
         <f>IFERROR((G12-F12)/F12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>RÉSULTAT D'EXPLOITATION</t>
         </is>
       </c>
-      <c r="B13" s="37">
+      <c r="B13" s="38">
         <f>B11+B12</f>
         <v/>
       </c>
-      <c r="C13" s="37">
+      <c r="C13" s="38">
         <f>C11+C12</f>
         <v/>
       </c>
-      <c r="D13" s="37">
+      <c r="D13" s="38">
         <f>D11+D12</f>
         <v/>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="39">
         <f>IFERROR((G13-F13)/F13,0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Marge EBITDA %</t>
         </is>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="40">
         <f>B11/B6</f>
         <v/>
       </c>
-      <c r="C14" s="39">
+      <c r="C14" s="40">
         <f>C11/C6</f>
         <v/>
       </c>
-      <c r="D14" s="39">
+      <c r="D14" s="40">
         <f>D11/D6</f>
         <v/>
       </c>
-      <c r="E14" s="40">
+      <c r="E14" s="41">
         <f>G14-F14</f>
         <v/>
       </c>
@@ -1670,7 +2312,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>À reproduire nativement : hiérarchie Compte + FST EBITDA. Colonne 2027 (V01/V02/V03) s'ajoute aux P&amp;L ②③④.</t>
         </is>
@@ -1725,346 +2367,346 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="43" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="43" t="inlineStr">
         <is>
           <t>→ Cand.</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="43" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E5" s="42" t="inlineStr">
+      <c r="E5" s="43" t="inlineStr">
         <is>
           <t>→ Admis</t>
         </is>
       </c>
-      <c r="F5" s="42" t="inlineStr">
+      <c r="F5" s="43" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G5" s="42" t="inlineStr">
+      <c r="G5" s="43" t="inlineStr">
         <is>
           <t>→ Inscrits</t>
         </is>
       </c>
-      <c r="H5" s="42" t="inlineStr">
+      <c r="H5" s="43" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="I5" s="42" t="inlineStr">
+      <c r="I5" s="43" t="inlineStr">
         <is>
           <t>Dépense acq.</t>
         </is>
       </c>
-      <c r="J5" s="42" t="inlineStr">
+      <c r="J5" s="43" t="inlineStr">
         <is>
           <t>CPL</t>
         </is>
       </c>
-      <c r="K5" s="42" t="inlineStr">
+      <c r="K5" s="43" t="inlineStr">
         <is>
           <t>CAC (€/inscrit)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Mbway</t>
         </is>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="44">
         <f>'Données CRM'!C15</f>
         <v/>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="44">
         <f>'Données CRM'!D15</f>
         <v/>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="45">
         <f>IFERROR('Données CRM'!D15/'Données CRM'!C15,0)</f>
         <v/>
       </c>
-      <c r="E6" s="43">
+      <c r="E6" s="44">
         <f>'Données CRM'!E15</f>
         <v/>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="45">
         <f>IFERROR('Données CRM'!E15/'Données CRM'!D15,0)</f>
         <v/>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="44">
         <f>'Données CRM'!F15</f>
         <v/>
       </c>
-      <c r="H6" s="44">
+      <c r="H6" s="45">
         <f>IFERROR('Données CRM'!F15/'Données CRM'!E15,0)</f>
         <v/>
       </c>
-      <c r="I6" s="43">
+      <c r="I6" s="44">
         <f>'Données CRM'!H15</f>
         <v/>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="44">
         <f>IFERROR('Données CRM'!H15/'Données CRM'!G15,0)</f>
         <v/>
       </c>
-      <c r="K6" s="43">
+      <c r="K6" s="44">
         <f>IFERROR('Données CRM'!H15/'Données CRM'!F15,0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Iscom</t>
         </is>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <f>'Données CRM'!C16</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <f>'Données CRM'!D16</f>
         <v/>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="18">
         <f>IFERROR('Données CRM'!D16/'Données CRM'!C16,0)</f>
         <v/>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="16">
         <f>'Données CRM'!E16</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="18">
         <f>IFERROR('Données CRM'!E16/'Données CRM'!D16,0)</f>
         <v/>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="16">
         <f>'Données CRM'!F16</f>
         <v/>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="18">
         <f>IFERROR('Données CRM'!F16/'Données CRM'!E16,0)</f>
         <v/>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="16">
         <f>'Données CRM'!H16</f>
         <v/>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="16">
         <f>IFERROR('Données CRM'!H16/'Données CRM'!G16,0)</f>
         <v/>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="16">
         <f>IFERROR('Données CRM'!H16/'Données CRM'!F16,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Ipac</t>
         </is>
       </c>
-      <c r="B8" s="43">
+      <c r="B8" s="44">
         <f>'Données CRM'!C17</f>
         <v/>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="44">
         <f>'Données CRM'!D17</f>
         <v/>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="45">
         <f>IFERROR('Données CRM'!D17/'Données CRM'!C17,0)</f>
         <v/>
       </c>
-      <c r="E8" s="43">
+      <c r="E8" s="44">
         <f>'Données CRM'!E17</f>
         <v/>
       </c>
-      <c r="F8" s="44">
+      <c r="F8" s="45">
         <f>IFERROR('Données CRM'!E17/'Données CRM'!D17,0)</f>
         <v/>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="44">
         <f>'Données CRM'!F17</f>
         <v/>
       </c>
-      <c r="H8" s="44">
+      <c r="H8" s="45">
         <f>IFERROR('Données CRM'!F17/'Données CRM'!E17,0)</f>
         <v/>
       </c>
-      <c r="I8" s="43">
+      <c r="I8" s="44">
         <f>'Données CRM'!H17</f>
         <v/>
       </c>
-      <c r="J8" s="43">
+      <c r="J8" s="44">
         <f>IFERROR('Données CRM'!H17/'Données CRM'!G17,0)</f>
         <v/>
       </c>
-      <c r="K8" s="43">
+      <c r="K8" s="44">
         <f>IFERROR('Données CRM'!H17/'Données CRM'!F17,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Pigier</t>
         </is>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="16">
         <f>'Données CRM'!C18</f>
         <v/>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="16">
         <f>'Données CRM'!D18</f>
         <v/>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="18">
         <f>IFERROR('Données CRM'!D18/'Données CRM'!C18,0)</f>
         <v/>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="16">
         <f>'Données CRM'!E18</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="18">
         <f>IFERROR('Données CRM'!E18/'Données CRM'!D18,0)</f>
         <v/>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="16">
         <f>'Données CRM'!F18</f>
         <v/>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="18">
         <f>IFERROR('Données CRM'!F18/'Données CRM'!E18,0)</f>
         <v/>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="16">
         <f>'Données CRM'!H18</f>
         <v/>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="16">
         <f>IFERROR('Données CRM'!H18/'Données CRM'!G18,0)</f>
         <v/>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="16">
         <f>IFERROR('Données CRM'!H18/'Données CRM'!F18,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="45" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>Tunon</t>
         </is>
       </c>
-      <c r="B10" s="43">
+      <c r="B10" s="44">
         <f>'Données CRM'!C19</f>
         <v/>
       </c>
-      <c r="C10" s="43">
+      <c r="C10" s="44">
         <f>'Données CRM'!D19</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="45">
         <f>IFERROR('Données CRM'!D19/'Données CRM'!C19,0)</f>
         <v/>
       </c>
-      <c r="E10" s="43">
+      <c r="E10" s="44">
         <f>'Données CRM'!E19</f>
         <v/>
       </c>
-      <c r="F10" s="44">
+      <c r="F10" s="45">
         <f>IFERROR('Données CRM'!E19/'Données CRM'!D19,0)</f>
         <v/>
       </c>
-      <c r="G10" s="43">
+      <c r="G10" s="44">
         <f>'Données CRM'!F19</f>
         <v/>
       </c>
-      <c r="H10" s="44">
+      <c r="H10" s="45">
         <f>IFERROR('Données CRM'!F19/'Données CRM'!E19,0)</f>
         <v/>
       </c>
-      <c r="I10" s="43">
+      <c r="I10" s="44">
         <f>'Données CRM'!H19</f>
         <v/>
       </c>
-      <c r="J10" s="43">
+      <c r="J10" s="44">
         <f>IFERROR('Données CRM'!H19/'Données CRM'!G19,0)</f>
         <v/>
       </c>
-      <c r="K10" s="46">
+      <c r="K10" s="47">
         <f>IFERROR('Données CRM'!H19/'Données CRM'!F19,0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>GROUPE</t>
         </is>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="49">
         <f>SUM(B6:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="49">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="49">
+      <c r="D11" s="50">
         <f>IFERROR(C11/B11,0)</f>
         <v/>
       </c>
-      <c r="E11" s="48">
+      <c r="E11" s="49">
         <f>SUM(E6:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="49">
+      <c r="F11" s="50">
         <f>IFERROR(E11/C11,0)</f>
         <v/>
       </c>
-      <c r="G11" s="48">
+      <c r="G11" s="49">
         <f>SUM(G6:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="49">
+      <c r="H11" s="50">
         <f>IFERROR(G11/E11,0)</f>
         <v/>
       </c>
-      <c r="I11" s="48">
+      <c r="I11" s="49">
         <f>SUM(I6:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="48">
+      <c r="J11" s="49">
         <f>IFERROR(I11/SUM('Données CRM'!G15:G19),0)</f>
         <v/>
       </c>
-      <c r="K11" s="48">
+      <c r="K11" s="49">
         <f>IFERROR(I11/G11,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="50" t="inlineStr">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>FIL ROUGE : Tunon ≈ 564 €/inscrit contre ~327 € MBway — même funnel, coût très supérieur → c'est LÀ qu'on agira (Acte 6).</t>
         </is>
@@ -2108,7 +2750,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>DONNÉES  ·  image de la vue V_PNL (VERSION = ACT, réel 2024-2026)</t>
         </is>
@@ -2122,752 +2764,752 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Compte</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Libellé</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>Nœud P&amp;L (FST)</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>Rôle allocation</t>
         </is>
       </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="E4" s="43" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="F4" s="43" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="52" t="inlineStr">
+      <c r="A5" s="53" t="inlineStr">
         <is>
           <t>706</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B5" s="54" t="inlineStr">
         <is>
           <t>Prestations de formation - scolarité (initial)</t>
         </is>
       </c>
-      <c r="C5" s="54" t="inlineStr">
+      <c r="C5" s="55" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="D5" s="54" t="inlineStr">
+      <c r="D5" s="55" t="inlineStr">
         <is>
           <t>PRODUIT</t>
         </is>
       </c>
-      <c r="E5" s="55" t="n">
+      <c r="E5" s="56" t="n">
         <v>2942930</v>
       </c>
-      <c r="F5" s="55" t="n">
+      <c r="F5" s="56" t="n">
         <v>3119504</v>
       </c>
-      <c r="G5" s="55" t="n">
+      <c r="G5" s="56" t="n">
         <v>3306675</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="56" t="inlineStr">
+      <c r="A6" s="57" t="inlineStr">
         <is>
           <t>7062</t>
         </is>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>Prestations de formation - alternance (OPCO)</t>
         </is>
       </c>
-      <c r="C6" s="58" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="D6" s="58" t="inlineStr">
+      <c r="D6" s="59" t="inlineStr">
         <is>
           <t>PRODUIT</t>
         </is>
       </c>
-      <c r="E6" s="59" t="n">
+      <c r="E6" s="60" t="n">
         <v>17023353</v>
       </c>
-      <c r="F6" s="59" t="n">
+      <c r="F6" s="60" t="n">
         <v>18044754</v>
       </c>
-      <c r="G6" s="59" t="n">
+      <c r="G6" s="60" t="n">
         <v>19127440</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="52" t="inlineStr">
+      <c r="A7" s="53" t="inlineStr">
         <is>
           <t>708</t>
         </is>
       </c>
-      <c r="B7" s="53" t="inlineStr">
+      <c r="B7" s="54" t="inlineStr">
         <is>
           <t>Frais de dossier &amp; droits d'inscription</t>
         </is>
       </c>
-      <c r="C7" s="54" t="inlineStr">
+      <c r="C7" s="55" t="inlineStr">
         <is>
           <t>PRODUITS</t>
         </is>
       </c>
-      <c r="D7" s="54" t="inlineStr">
+      <c r="D7" s="55" t="inlineStr">
         <is>
           <t>PRODUIT</t>
         </is>
       </c>
-      <c r="E7" s="55" t="n">
+      <c r="E7" s="56" t="n">
         <v>98442</v>
       </c>
-      <c r="F7" s="55" t="n">
+      <c r="F7" s="56" t="n">
         <v>104348</v>
       </c>
-      <c r="G7" s="55" t="n">
+      <c r="G7" s="56" t="n">
         <v>110610</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="56" t="inlineStr">
+      <c r="A8" s="57" t="inlineStr">
         <is>
           <t>604</t>
         </is>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>Sous-traitance pédagogique</t>
         </is>
       </c>
-      <c r="C8" s="58" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
           <t>COUTS_DIRECTS</t>
         </is>
       </c>
-      <c r="D8" s="58" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
       </c>
-      <c r="E8" s="59" t="n">
+      <c r="E8" s="60" t="n">
         <v>618583</v>
       </c>
-      <c r="F8" s="59" t="n">
+      <c r="F8" s="60" t="n">
         <v>646928</v>
       </c>
-      <c r="G8" s="59" t="n">
+      <c r="G8" s="60" t="n">
         <v>677808</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="52" t="inlineStr">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>6063</t>
         </is>
       </c>
-      <c r="B9" s="53" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>Fournitures pédagogiques &amp; petit équipement</t>
         </is>
       </c>
-      <c r="C9" s="54" t="inlineStr">
+      <c r="C9" s="55" t="inlineStr">
         <is>
           <t>COUTS_DIRECTS</t>
         </is>
       </c>
-      <c r="D9" s="54" t="inlineStr">
+      <c r="D9" s="55" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
       </c>
-      <c r="E9" s="55" t="n">
+      <c r="E9" s="56" t="n">
         <v>412387</v>
       </c>
-      <c r="F9" s="55" t="n">
+      <c r="F9" s="56" t="n">
         <v>431286</v>
       </c>
-      <c r="G9" s="55" t="n">
+      <c r="G9" s="56" t="n">
         <v>451874</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="56" t="inlineStr">
+      <c r="A10" s="57" t="inlineStr">
         <is>
           <t>621</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>Personnel extérieur - vacataires</t>
         </is>
       </c>
-      <c r="C10" s="58" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
           <t>COUTS_DIRECTS</t>
         </is>
       </c>
-      <c r="D10" s="58" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
       </c>
-      <c r="E10" s="59" t="n">
+      <c r="E10" s="60" t="n">
         <v>1443361</v>
       </c>
-      <c r="F10" s="59" t="n">
+      <c r="F10" s="60" t="n">
         <v>1509499</v>
       </c>
-      <c r="G10" s="59" t="n">
+      <c r="G10" s="60" t="n">
         <v>1581554</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="52" t="inlineStr">
+      <c r="A11" s="53" t="inlineStr">
         <is>
           <t>6231</t>
         </is>
       </c>
-      <c r="B11" s="53" t="inlineStr">
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>Publicité &amp; marketing d'acquisition</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C11" s="55" t="inlineStr">
         <is>
           <t>COUTS_DIRECTS</t>
         </is>
       </c>
-      <c r="D11" s="54" t="inlineStr">
+      <c r="D11" s="55" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
       </c>
-      <c r="E11" s="55" t="n">
+      <c r="E11" s="56" t="n">
         <v>358819</v>
       </c>
-      <c r="F11" s="55" t="n">
+      <c r="F11" s="56" t="n">
         <v>394702</v>
       </c>
-      <c r="G11" s="55" t="n">
+      <c r="G11" s="56" t="n">
         <v>434174</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="56" t="inlineStr">
+      <c r="A12" s="57" t="inlineStr">
         <is>
           <t>6411</t>
         </is>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="58" t="inlineStr">
         <is>
           <t>Rémunération enseignants permanents</t>
         </is>
       </c>
-      <c r="C12" s="58" t="inlineStr">
+      <c r="C12" s="59" t="inlineStr">
         <is>
           <t>PERSONNEL</t>
         </is>
       </c>
-      <c r="D12" s="58" t="inlineStr">
+      <c r="D12" s="59" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
       </c>
-      <c r="E12" s="59" t="n">
+      <c r="E12" s="60" t="n">
         <v>3505311</v>
       </c>
-      <c r="F12" s="59" t="n">
+      <c r="F12" s="60" t="n">
         <v>3665931</v>
       </c>
-      <c r="G12" s="59" t="n">
+      <c r="G12" s="60" t="n">
         <v>3840917</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="52" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t>6413</t>
         </is>
       </c>
-      <c r="B13" s="53" t="inlineStr">
+      <c r="B13" s="54" t="inlineStr">
         <is>
           <t>Rémunération personnel administratif</t>
         </is>
       </c>
-      <c r="C13" s="54" t="inlineStr">
+      <c r="C13" s="55" t="inlineStr">
         <is>
           <t>PERSONNEL</t>
         </is>
       </c>
-      <c r="D13" s="54" t="inlineStr">
+      <c r="D13" s="55" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E13" s="55" t="n">
+      <c r="E13" s="56" t="n">
         <v>1855752</v>
       </c>
-      <c r="F13" s="55" t="n">
+      <c r="F13" s="56" t="n">
         <v>1940786</v>
       </c>
-      <c r="G13" s="55" t="n">
+      <c r="G13" s="56" t="n">
         <v>2033426</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="56" t="inlineStr">
+      <c r="A14" s="57" t="inlineStr">
         <is>
           <t>6414</t>
         </is>
       </c>
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t>Rémunération direction &amp; siège</t>
         </is>
       </c>
-      <c r="C14" s="58" t="inlineStr">
+      <c r="C14" s="59" t="inlineStr">
         <is>
           <t>PERSONNEL</t>
         </is>
       </c>
-      <c r="D14" s="58" t="inlineStr">
+      <c r="D14" s="59" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E14" s="59" t="n">
+      <c r="E14" s="60" t="n">
         <v>1134071</v>
       </c>
-      <c r="F14" s="59" t="n">
+      <c r="F14" s="60" t="n">
         <v>1186037</v>
       </c>
-      <c r="G14" s="59" t="n">
+      <c r="G14" s="60" t="n">
         <v>1242649</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="52" t="inlineStr">
+      <c r="A15" s="53" t="inlineStr">
         <is>
           <t>645</t>
         </is>
       </c>
-      <c r="B15" s="53" t="inlineStr">
+      <c r="B15" s="54" t="inlineStr">
         <is>
           <t>Charges sociales &amp; prévoyance</t>
         </is>
       </c>
-      <c r="C15" s="54" t="inlineStr">
+      <c r="C15" s="55" t="inlineStr">
         <is>
           <t>PERSONNEL</t>
         </is>
       </c>
-      <c r="D15" s="54" t="inlineStr">
+      <c r="D15" s="55" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E15" s="55" t="n">
+      <c r="E15" s="56" t="n">
         <v>2886726</v>
       </c>
-      <c r="F15" s="55" t="n">
+      <c r="F15" s="56" t="n">
         <v>3019002</v>
       </c>
-      <c r="G15" s="55" t="n">
+      <c r="G15" s="56" t="n">
         <v>3163106</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="56" t="inlineStr">
+      <c r="A16" s="57" t="inlineStr">
         <is>
           <t>613</t>
         </is>
       </c>
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t>Loyers &amp; charges locatives</t>
         </is>
       </c>
-      <c r="C16" s="58" t="inlineStr">
+      <c r="C16" s="59" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D16" s="58" t="inlineStr">
+      <c r="D16" s="59" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E16" s="59" t="n">
+      <c r="E16" s="60" t="n">
         <v>2165045</v>
       </c>
-      <c r="F16" s="59" t="n">
+      <c r="F16" s="60" t="n">
         <v>2264254</v>
       </c>
-      <c r="G16" s="59" t="n">
+      <c r="G16" s="60" t="n">
         <v>2372329</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="52" t="inlineStr">
+      <c r="A17" s="53" t="inlineStr">
         <is>
           <t>615</t>
         </is>
       </c>
-      <c r="B17" s="53" t="inlineStr">
+      <c r="B17" s="54" t="inlineStr">
         <is>
           <t>Entretien &amp; maintenance</t>
         </is>
       </c>
-      <c r="C17" s="54" t="inlineStr">
+      <c r="C17" s="55" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D17" s="54" t="inlineStr">
+      <c r="D17" s="55" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E17" s="55" t="n">
+      <c r="E17" s="56" t="n">
         <v>309291</v>
       </c>
-      <c r="F17" s="55" t="n">
+      <c r="F17" s="56" t="n">
         <v>323463</v>
       </c>
-      <c r="G17" s="55" t="n">
+      <c r="G17" s="56" t="n">
         <v>338902</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="56" t="inlineStr">
+      <c r="A18" s="57" t="inlineStr">
         <is>
           <t>616</t>
         </is>
       </c>
-      <c r="B18" s="57" t="inlineStr">
+      <c r="B18" s="58" t="inlineStr">
         <is>
           <t>Primes d'assurance</t>
         </is>
       </c>
-      <c r="C18" s="58" t="inlineStr">
+      <c r="C18" s="59" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D18" s="58" t="inlineStr">
+      <c r="D18" s="59" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E18" s="59" t="n">
+      <c r="E18" s="60" t="n">
         <v>206194</v>
       </c>
-      <c r="F18" s="59" t="n">
+      <c r="F18" s="60" t="n">
         <v>215645</v>
       </c>
-      <c r="G18" s="59" t="n">
+      <c r="G18" s="60" t="n">
         <v>225937</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="52" t="inlineStr">
+      <c r="A19" s="53" t="inlineStr">
         <is>
           <t>6226</t>
         </is>
       </c>
-      <c r="B19" s="53" t="inlineStr">
+      <c r="B19" s="54" t="inlineStr">
         <is>
           <t>Honoraires</t>
         </is>
       </c>
-      <c r="C19" s="54" t="inlineStr">
+      <c r="C19" s="55" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D19" s="54" t="inlineStr">
+      <c r="D19" s="55" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E19" s="55" t="n">
+      <c r="E19" s="56" t="n">
         <v>515487</v>
       </c>
-      <c r="F19" s="55" t="n">
+      <c r="F19" s="56" t="n">
         <v>539108</v>
       </c>
-      <c r="G19" s="55" t="n">
+      <c r="G19" s="56" t="n">
         <v>564841</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="56" t="inlineStr">
+      <c r="A20" s="57" t="inlineStr">
         <is>
           <t>6236</t>
         </is>
       </c>
-      <c r="B20" s="57" t="inlineStr">
+      <c r="B20" s="58" t="inlineStr">
         <is>
           <t>Marketing de marque, salons &amp; JPO</t>
         </is>
       </c>
-      <c r="C20" s="58" t="inlineStr">
+      <c r="C20" s="59" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D20" s="58" t="inlineStr">
+      <c r="D20" s="59" t="inlineStr">
         <is>
           <t>FRAIS_MARQUE</t>
         </is>
       </c>
-      <c r="E20" s="59" t="n">
+      <c r="E20" s="60" t="n">
         <v>499926</v>
       </c>
-      <c r="F20" s="59" t="n">
+      <c r="F20" s="60" t="n">
         <v>580167</v>
       </c>
-      <c r="G20" s="59" t="n">
+      <c r="G20" s="60" t="n">
         <v>676344</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="52" t="inlineStr">
+      <c r="A21" s="53" t="inlineStr">
         <is>
           <t>625</t>
         </is>
       </c>
-      <c r="B21" s="53" t="inlineStr">
+      <c r="B21" s="54" t="inlineStr">
         <is>
           <t>Déplacements &amp; missions</t>
         </is>
       </c>
-      <c r="C21" s="54" t="inlineStr">
+      <c r="C21" s="55" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D21" s="54" t="inlineStr">
+      <c r="D21" s="55" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E21" s="55" t="n">
+      <c r="E21" s="56" t="n">
         <v>309292</v>
       </c>
-      <c r="F21" s="55" t="n">
+      <c r="F21" s="56" t="n">
         <v>323464</v>
       </c>
-      <c r="G21" s="55" t="n">
+      <c r="G21" s="56" t="n">
         <v>338906</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="56" t="inlineStr">
+      <c r="A22" s="57" t="inlineStr">
         <is>
           <t>626</t>
         </is>
       </c>
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="58" t="inlineStr">
         <is>
           <t>Télécom &amp; SI</t>
         </is>
       </c>
-      <c r="C22" s="58" t="inlineStr">
+      <c r="C22" s="59" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D22" s="58" t="inlineStr">
+      <c r="D22" s="59" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E22" s="59" t="n">
+      <c r="E22" s="60" t="n">
         <v>412389</v>
       </c>
-      <c r="F22" s="59" t="n">
+      <c r="F22" s="60" t="n">
         <v>431286</v>
       </c>
-      <c r="G22" s="59" t="n">
+      <c r="G22" s="60" t="n">
         <v>451872</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="52" t="inlineStr">
+      <c r="A23" s="53" t="inlineStr">
         <is>
           <t>6281</t>
         </is>
       </c>
-      <c r="B23" s="53" t="inlineStr">
+      <c r="B23" s="54" t="inlineStr">
         <is>
           <t>Cotisations &amp; abonnements</t>
         </is>
       </c>
-      <c r="C23" s="54" t="inlineStr">
+      <c r="C23" s="55" t="inlineStr">
         <is>
           <t>STRUCTURE</t>
         </is>
       </c>
-      <c r="D23" s="54" t="inlineStr">
+      <c r="D23" s="55" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E23" s="55" t="n">
+      <c r="E23" s="56" t="n">
         <v>164956</v>
       </c>
-      <c r="F23" s="55" t="n">
+      <c r="F23" s="56" t="n">
         <v>172514</v>
       </c>
-      <c r="G23" s="55" t="n">
+      <c r="G23" s="56" t="n">
         <v>180749</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="56" t="inlineStr">
+      <c r="A24" s="57" t="inlineStr">
         <is>
           <t>6331</t>
         </is>
       </c>
-      <c r="B24" s="57" t="inlineStr">
+      <c r="B24" s="58" t="inlineStr">
         <is>
           <t>Taxe sur les salaires</t>
         </is>
       </c>
-      <c r="C24" s="58" t="inlineStr">
+      <c r="C24" s="59" t="inlineStr">
         <is>
           <t>IMPOTS_TAXES</t>
         </is>
       </c>
-      <c r="D24" s="58" t="inlineStr">
+      <c r="D24" s="59" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E24" s="59" t="n">
+      <c r="E24" s="60" t="n">
         <v>309292</v>
       </c>
-      <c r="F24" s="59" t="n">
+      <c r="F24" s="60" t="n">
         <v>323465</v>
       </c>
-      <c r="G24" s="59" t="n">
+      <c r="G24" s="60" t="n">
         <v>338904</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="52" t="inlineStr">
+      <c r="A25" s="53" t="inlineStr">
         <is>
           <t>6333</t>
         </is>
       </c>
-      <c r="B25" s="53" t="inlineStr">
+      <c r="B25" s="54" t="inlineStr">
         <is>
           <t>Participation formation</t>
         </is>
       </c>
-      <c r="C25" s="54" t="inlineStr">
+      <c r="C25" s="55" t="inlineStr">
         <is>
           <t>IMPOTS_TAXES</t>
         </is>
       </c>
-      <c r="D25" s="54" t="inlineStr">
+      <c r="D25" s="55" t="inlineStr">
         <is>
           <t>HOLDING</t>
         </is>
       </c>
-      <c r="E25" s="55" t="n">
+      <c r="E25" s="56" t="n">
         <v>103097</v>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="56" t="n">
         <v>107822</v>
       </c>
-      <c r="G25" s="55" t="n">
+      <c r="G25" s="56" t="n">
         <v>112968</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="A26" s="57" t="inlineStr">
         <is>
           <t>63511</t>
         </is>
       </c>
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B26" s="58" t="inlineStr">
         <is>
           <t>Cotisation foncière &amp; CVAE</t>
         </is>
       </c>
-      <c r="C26" s="58" t="inlineStr">
+      <c r="C26" s="59" t="inlineStr">
         <is>
           <t>IMPOTS_TAXES</t>
         </is>
       </c>
-      <c r="D26" s="58" t="inlineStr">
+      <c r="D26" s="59" t="inlineStr">
         <is>
           <t>STRUCT_CAMP</t>
         </is>
       </c>
-      <c r="E26" s="59" t="n">
+      <c r="E26" s="60" t="n">
         <v>206196</v>
       </c>
-      <c r="F26" s="59" t="n">
+      <c r="F26" s="60" t="n">
         <v>215643</v>
       </c>
-      <c r="G26" s="59" t="n">
+      <c r="G26" s="60" t="n">
         <v>225935</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="52" t="inlineStr">
+      <c r="A27" s="53" t="inlineStr">
         <is>
           <t>6811</t>
         </is>
       </c>
-      <c r="B27" s="53" t="inlineStr">
+      <c r="B27" s="54" t="inlineStr">
         <is>
           <t>Dotations aux amortissements</t>
         </is>
       </c>
-      <c r="C27" s="54" t="inlineStr">
+      <c r="C27" s="55" t="inlineStr">
         <is>
           <t>DOTATIONS</t>
         </is>
       </c>
-      <c r="D27" s="54" t="inlineStr">
+      <c r="D27" s="55" t="inlineStr">
         <is>
           <t>DOTATION</t>
         </is>
       </c>
-      <c r="E27" s="55" t="n">
+      <c r="E27" s="56" t="n">
         <v>1203886</v>
       </c>
-      <c r="F27" s="55" t="n">
+      <c r="F27" s="56" t="n">
         <v>1276115</v>
       </c>
-      <c r="G27" s="55" t="n">
+      <c r="G27" s="56" t="n">
         <v>1352683</v>
       </c>
     </row>
@@ -2896,7 +3538,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="51" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>DONNÉES  ·  image des vues V_FUNNEL + V_CAC (socle CRM)</t>
         </is>
@@ -2910,494 +3552,494 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Exercice</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Marque</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="43" t="inlineStr">
         <is>
           <t>Leads</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="43" t="inlineStr">
         <is>
           <t>Candidats</t>
         </is>
       </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="E4" s="43" t="inlineStr">
         <is>
           <t>Admis</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="F4" s="43" t="inlineStr">
         <is>
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="43" t="inlineStr">
         <is>
           <t>Leads payants</t>
         </is>
       </c>
-      <c r="H4" s="42" t="inlineStr">
+      <c r="H4" s="43" t="inlineStr">
         <is>
           <t>Dépense acq. (€)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="60" t="inlineStr">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B5" s="54" t="inlineStr">
         <is>
           <t>MBWAY</t>
         </is>
       </c>
-      <c r="C5" s="55" t="n">
+      <c r="C5" s="56" t="n">
         <v>5736</v>
       </c>
-      <c r="D5" s="55" t="n">
+      <c r="D5" s="56" t="n">
         <v>1298</v>
       </c>
-      <c r="E5" s="55" t="n">
+      <c r="E5" s="56" t="n">
         <v>920</v>
       </c>
-      <c r="F5" s="55" t="n">
+      <c r="F5" s="56" t="n">
         <v>452</v>
       </c>
-      <c r="G5" s="55" t="n">
+      <c r="G5" s="56" t="n">
         <v>3326</v>
       </c>
-      <c r="H5" s="55" t="n">
+      <c r="H5" s="56" t="n">
         <v>137627</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="61" t="inlineStr">
+      <c r="A6" s="62" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C6" s="59" t="n">
+      <c r="C6" s="60" t="n">
         <v>3794</v>
       </c>
-      <c r="D6" s="59" t="n">
+      <c r="D6" s="60" t="n">
         <v>857</v>
       </c>
-      <c r="E6" s="59" t="n">
+      <c r="E6" s="60" t="n">
         <v>608</v>
       </c>
-      <c r="F6" s="59" t="n">
+      <c r="F6" s="60" t="n">
         <v>300</v>
       </c>
-      <c r="G6" s="59" t="n">
+      <c r="G6" s="60" t="n">
         <v>2132</v>
       </c>
-      <c r="H6" s="59" t="n">
+      <c r="H6" s="60" t="n">
         <v>89342</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="60" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B7" s="53" t="inlineStr">
+      <c r="B7" s="54" t="inlineStr">
         <is>
           <t>IPAC</t>
         </is>
       </c>
-      <c r="C7" s="55" t="n">
+      <c r="C7" s="56" t="n">
         <v>1966</v>
       </c>
-      <c r="D7" s="55" t="n">
+      <c r="D7" s="56" t="n">
         <v>393</v>
       </c>
-      <c r="E7" s="55" t="n">
+      <c r="E7" s="56" t="n">
         <v>276</v>
       </c>
-      <c r="F7" s="55" t="n">
+      <c r="F7" s="56" t="n">
         <v>116</v>
       </c>
-      <c r="G7" s="55" t="n">
+      <c r="G7" s="56" t="n">
         <v>1237</v>
       </c>
-      <c r="H7" s="55" t="n">
+      <c r="H7" s="56" t="n">
         <v>42867</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="62" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>PIGIER</t>
         </is>
       </c>
-      <c r="C8" s="59" t="n">
+      <c r="C8" s="60" t="n">
         <v>2492</v>
       </c>
-      <c r="D8" s="59" t="n">
+      <c r="D8" s="60" t="n">
         <v>498</v>
       </c>
-      <c r="E8" s="59" t="n">
+      <c r="E8" s="60" t="n">
         <v>350</v>
       </c>
-      <c r="F8" s="59" t="n">
+      <c r="F8" s="60" t="n">
         <v>146</v>
       </c>
-      <c r="G8" s="59" t="n">
+      <c r="G8" s="60" t="n">
         <v>1293</v>
       </c>
-      <c r="H8" s="59" t="n">
+      <c r="H8" s="60" t="n">
         <v>48413</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="60" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B9" s="53" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>TUNON</t>
         </is>
       </c>
-      <c r="C9" s="55" t="n">
+      <c r="C9" s="56" t="n">
         <v>1317</v>
       </c>
-      <c r="D9" s="55" t="n">
+      <c r="D9" s="56" t="n">
         <v>263</v>
       </c>
-      <c r="E9" s="55" t="n">
+      <c r="E9" s="56" t="n">
         <v>185</v>
       </c>
-      <c r="F9" s="55" t="n">
+      <c r="F9" s="56" t="n">
         <v>78</v>
       </c>
-      <c r="G9" s="55" t="n">
+      <c r="G9" s="56" t="n">
         <v>909</v>
       </c>
-      <c r="H9" s="55" t="n">
+      <c r="H9" s="56" t="n">
         <v>40570</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="62" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>MBWAY</t>
         </is>
       </c>
-      <c r="C10" s="59" t="n">
+      <c r="C10" s="60" t="n">
         <v>6079</v>
       </c>
-      <c r="D10" s="59" t="n">
+      <c r="D10" s="60" t="n">
         <v>1374</v>
       </c>
-      <c r="E10" s="59" t="n">
+      <c r="E10" s="60" t="n">
         <v>973</v>
       </c>
-      <c r="F10" s="59" t="n">
+      <c r="F10" s="60" t="n">
         <v>482</v>
       </c>
-      <c r="G10" s="59" t="n">
+      <c r="G10" s="60" t="n">
         <v>3487</v>
       </c>
-      <c r="H10" s="59" t="n">
+      <c r="H10" s="60" t="n">
         <v>151390</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="60" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B11" s="53" t="inlineStr">
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C11" s="55" t="n">
+      <c r="C11" s="56" t="n">
         <v>4022</v>
       </c>
-      <c r="D11" s="55" t="n">
+      <c r="D11" s="56" t="n">
         <v>909</v>
       </c>
-      <c r="E11" s="55" t="n">
+      <c r="E11" s="56" t="n">
         <v>644</v>
       </c>
-      <c r="F11" s="55" t="n">
+      <c r="F11" s="56" t="n">
         <v>318</v>
       </c>
-      <c r="G11" s="55" t="n">
+      <c r="G11" s="56" t="n">
         <v>2233</v>
       </c>
-      <c r="H11" s="55" t="n">
+      <c r="H11" s="56" t="n">
         <v>98275</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="62" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="58" t="inlineStr">
         <is>
           <t>IPAC</t>
         </is>
       </c>
-      <c r="C12" s="59" t="n">
+      <c r="C12" s="60" t="n">
         <v>2086</v>
       </c>
-      <c r="D12" s="59" t="n">
+      <c r="D12" s="60" t="n">
         <v>416</v>
       </c>
-      <c r="E12" s="59" t="n">
+      <c r="E12" s="60" t="n">
         <v>292</v>
       </c>
-      <c r="F12" s="59" t="n">
+      <c r="F12" s="60" t="n">
         <v>123</v>
       </c>
-      <c r="G12" s="59" t="n">
+      <c r="G12" s="60" t="n">
         <v>1307</v>
       </c>
-      <c r="H12" s="59" t="n">
+      <c r="H12" s="60" t="n">
         <v>47155</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="60" t="inlineStr">
+      <c r="A13" s="61" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B13" s="53" t="inlineStr">
+      <c r="B13" s="54" t="inlineStr">
         <is>
           <t>PIGIER</t>
         </is>
       </c>
-      <c r="C13" s="55" t="n">
+      <c r="C13" s="56" t="n">
         <v>2642</v>
       </c>
-      <c r="D13" s="55" t="n">
+      <c r="D13" s="56" t="n">
         <v>528</v>
       </c>
-      <c r="E13" s="55" t="n">
+      <c r="E13" s="56" t="n">
         <v>370</v>
       </c>
-      <c r="F13" s="55" t="n">
+      <c r="F13" s="56" t="n">
         <v>154</v>
       </c>
-      <c r="G13" s="55" t="n">
+      <c r="G13" s="56" t="n">
         <v>1350</v>
       </c>
-      <c r="H13" s="55" t="n">
+      <c r="H13" s="56" t="n">
         <v>53255</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr">
+      <c r="A14" s="62" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t>TUNON</t>
         </is>
       </c>
-      <c r="C14" s="59" t="n">
+      <c r="C14" s="60" t="n">
         <v>1397</v>
       </c>
-      <c r="D14" s="59" t="n">
+      <c r="D14" s="60" t="n">
         <v>279</v>
       </c>
-      <c r="E14" s="59" t="n">
+      <c r="E14" s="60" t="n">
         <v>196</v>
       </c>
-      <c r="F14" s="59" t="n">
+      <c r="F14" s="60" t="n">
         <v>82</v>
       </c>
-      <c r="G14" s="59" t="n">
+      <c r="G14" s="60" t="n">
         <v>948</v>
       </c>
-      <c r="H14" s="59" t="n">
+      <c r="H14" s="60" t="n">
         <v>44627</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="60" t="inlineStr">
+      <c r="A15" s="61" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B15" s="53" t="inlineStr">
+      <c r="B15" s="54" t="inlineStr">
         <is>
           <t>MBWAY</t>
         </is>
       </c>
-      <c r="C15" s="55" t="n">
+      <c r="C15" s="56" t="n">
         <v>6444</v>
       </c>
-      <c r="D15" s="55" t="n">
+      <c r="D15" s="56" t="n">
         <v>1458</v>
       </c>
-      <c r="E15" s="55" t="n">
+      <c r="E15" s="56" t="n">
         <v>1032</v>
       </c>
-      <c r="F15" s="55" t="n">
+      <c r="F15" s="56" t="n">
         <v>510</v>
       </c>
-      <c r="G15" s="55" t="n">
+      <c r="G15" s="56" t="n">
         <v>3659</v>
       </c>
-      <c r="H15" s="55" t="n">
+      <c r="H15" s="56" t="n">
         <v>166530</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="61" t="inlineStr">
+      <c r="A16" s="62" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="C16" s="59" t="n">
+      <c r="C16" s="60" t="n">
         <v>4263</v>
       </c>
-      <c r="D16" s="59" t="n">
+      <c r="D16" s="60" t="n">
         <v>964</v>
       </c>
-      <c r="E16" s="59" t="n">
+      <c r="E16" s="60" t="n">
         <v>683</v>
       </c>
-      <c r="F16" s="59" t="n">
+      <c r="F16" s="60" t="n">
         <v>338</v>
       </c>
-      <c r="G16" s="59" t="n">
+      <c r="G16" s="60" t="n">
         <v>2337</v>
       </c>
-      <c r="H16" s="59" t="n">
+      <c r="H16" s="60" t="n">
         <v>108103</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="60" t="inlineStr">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B17" s="53" t="inlineStr">
+      <c r="B17" s="54" t="inlineStr">
         <is>
           <t>IPAC</t>
         </is>
       </c>
-      <c r="C17" s="55" t="n">
+      <c r="C17" s="56" t="n">
         <v>2210</v>
       </c>
-      <c r="D17" s="55" t="n">
+      <c r="D17" s="56" t="n">
         <v>442</v>
       </c>
-      <c r="E17" s="55" t="n">
+      <c r="E17" s="56" t="n">
         <v>309</v>
       </c>
-      <c r="F17" s="55" t="n">
+      <c r="F17" s="56" t="n">
         <v>130</v>
       </c>
-      <c r="G17" s="55" t="n">
+      <c r="G17" s="56" t="n">
         <v>1381</v>
       </c>
-      <c r="H17" s="55" t="n">
+      <c r="H17" s="56" t="n">
         <v>51871</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="61" t="inlineStr">
+      <c r="A18" s="62" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B18" s="57" t="inlineStr">
+      <c r="B18" s="58" t="inlineStr">
         <is>
           <t>PIGIER</t>
         </is>
       </c>
-      <c r="C18" s="59" t="n">
+      <c r="C18" s="60" t="n">
         <v>2800</v>
       </c>
-      <c r="D18" s="59" t="n">
+      <c r="D18" s="60" t="n">
         <v>560</v>
       </c>
-      <c r="E18" s="59" t="n">
+      <c r="E18" s="60" t="n">
         <v>392</v>
       </c>
-      <c r="F18" s="59" t="n">
+      <c r="F18" s="60" t="n">
         <v>164</v>
       </c>
-      <c r="G18" s="59" t="n">
+      <c r="G18" s="60" t="n">
         <v>1410</v>
       </c>
-      <c r="H18" s="59" t="n">
+      <c r="H18" s="60" t="n">
         <v>58580</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="60" t="inlineStr">
+      <c r="A19" s="61" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B19" s="53" t="inlineStr">
+      <c r="B19" s="54" t="inlineStr">
         <is>
           <t>TUNON</t>
         </is>
       </c>
-      <c r="C19" s="55" t="n">
+      <c r="C19" s="56" t="n">
         <v>1480</v>
       </c>
-      <c r="D19" s="55" t="n">
+      <c r="D19" s="56" t="n">
         <v>296</v>
       </c>
-      <c r="E19" s="55" t="n">
+      <c r="E19" s="56" t="n">
         <v>207</v>
       </c>
-      <c r="F19" s="55" t="n">
+      <c r="F19" s="56" t="n">
         <v>87</v>
       </c>
-      <c r="G19" s="55" t="n">
+      <c r="G19" s="56" t="n">
         <v>988</v>
       </c>
-      <c r="H19" s="55" t="n">
+      <c r="H19" s="56" t="n">
         <v>49090</v>
       </c>
     </row>

</xml_diff>